<commit_message>
Sync new character resources and item icons from Tencent sheets
</commit_message>
<xml_diff>
--- a/Excel/CharacterPart.xlsx
+++ b/Excel/CharacterPart.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t/>
   </si>
@@ -230,6 +230,18 @@
   </si>
   <si>
     <t>float</t>
+  </si>
+  <si>
+    <t>character_c_walk_body_01</t>
+  </si>
+  <si>
+    <t>character_c_walk_face_01</t>
+  </si>
+  <si>
+    <t>character_c_walk_hair_01</t>
+  </si>
+  <si>
+    <t>character_c_walk_hair_03</t>
   </si>
 </sst>
 </file>
@@ -359,7 +371,7 @@
     <xf numFmtId="301" fontId="9" fillId="0" borderId="3" xfId="0"/>
     <xf numFmtId="301" fontId="9" fillId="4" borderId="3" xfId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -452,6 +464,7 @@
     <xf numFmtId="49" fontId="6" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -656,7 +669,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="J219"/>
+  <dimension ref="J243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.7109" customWidth="1"/>
@@ -4672,6 +4685,438 @@
       <c r="I219" s="17" t="s"/>
       <c r="J219" s="13" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="220" spans="1:10" ht="24" customHeight="1">
+      <c r="A220" s="9" t="s"/>
+      <c r="B220" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C220" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D220" s="11" t="s"/>
+      <c r="E220" s="24" t="s"/>
+      <c r="F220" s="11" t="s"/>
+      <c r="G220" s="24" t="s"/>
+      <c r="H220" s="11" t="s"/>
+      <c r="I220" s="24" t="s"/>
+      <c r="J220" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="221" spans="1:10" ht="24" customHeight="1">
+      <c r="A221" s="18" t="s"/>
+      <c r="B221" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C221" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D221" s="11" t="s"/>
+      <c r="E221" s="24" t="s"/>
+      <c r="F221" s="11" t="s"/>
+      <c r="G221" s="24" t="s"/>
+      <c r="H221" s="11" t="s"/>
+      <c r="I221" s="24" t="s"/>
+      <c r="J221" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="222" spans="1:10" ht="24" customHeight="1">
+      <c r="A222" s="18" t="s"/>
+      <c r="B222" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C222" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D222" s="11" t="s"/>
+      <c r="E222" s="24" t="s"/>
+      <c r="F222" s="11" t="s"/>
+      <c r="G222" s="24" t="s"/>
+      <c r="H222" s="11" t="s"/>
+      <c r="I222" s="24" t="s"/>
+      <c r="J222" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="223" spans="1:10" ht="24" customHeight="1">
+      <c r="A223" s="18" t="s"/>
+      <c r="B223" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C223" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D223" s="11" t="s"/>
+      <c r="E223" s="24" t="s"/>
+      <c r="F223" s="11" t="s"/>
+      <c r="G223" s="24" t="s"/>
+      <c r="H223" s="11" t="s"/>
+      <c r="I223" s="24" t="s"/>
+      <c r="J223" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="224" spans="1:10" ht="24" customHeight="1">
+      <c r="A224" s="18" t="s"/>
+      <c r="B224" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C224" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D224" s="11" t="s"/>
+      <c r="E224" s="24" t="s"/>
+      <c r="F224" s="11" t="s"/>
+      <c r="G224" s="24" t="s"/>
+      <c r="H224" s="11" t="s"/>
+      <c r="I224" s="24" t="s"/>
+      <c r="J224" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="225" spans="1:10" ht="24" customHeight="1">
+      <c r="A225" s="18" t="s"/>
+      <c r="B225" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C225" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D225" s="11" t="s"/>
+      <c r="E225" s="24" t="s"/>
+      <c r="F225" s="11" t="s"/>
+      <c r="G225" s="24" t="s"/>
+      <c r="H225" s="11" t="s"/>
+      <c r="I225" s="24" t="s"/>
+      <c r="J225" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="226" spans="1:10" ht="24" customHeight="1">
+      <c r="A226" s="9" t="s"/>
+      <c r="B226" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C226" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D226" s="11" t="s"/>
+      <c r="E226" s="24" t="s"/>
+      <c r="F226" s="11" t="s"/>
+      <c r="G226" s="24" t="s"/>
+      <c r="H226" s="11" t="s"/>
+      <c r="I226" s="24" t="s"/>
+      <c r="J226" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="227" spans="1:10" ht="24" customHeight="1">
+      <c r="A227" s="18" t="s"/>
+      <c r="B227" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C227" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D227" s="11" t="s"/>
+      <c r="E227" s="24" t="s"/>
+      <c r="F227" s="11" t="s"/>
+      <c r="G227" s="24" t="s"/>
+      <c r="H227" s="11" t="s"/>
+      <c r="I227" s="24" t="s"/>
+      <c r="J227" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="228" spans="1:10" ht="24" customHeight="1">
+      <c r="A228" s="18" t="s"/>
+      <c r="B228" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C228" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D228" s="11" t="s"/>
+      <c r="E228" s="24" t="s"/>
+      <c r="F228" s="11" t="s"/>
+      <c r="G228" s="24" t="s"/>
+      <c r="H228" s="11" t="s"/>
+      <c r="I228" s="24" t="s"/>
+      <c r="J228" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="229" spans="1:10" ht="24" customHeight="1">
+      <c r="A229" s="18" t="s"/>
+      <c r="B229" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C229" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D229" s="11" t="s"/>
+      <c r="E229" s="24" t="s"/>
+      <c r="F229" s="11" t="s"/>
+      <c r="G229" s="24" t="s"/>
+      <c r="H229" s="11" t="s"/>
+      <c r="I229" s="24" t="s"/>
+      <c r="J229" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="230" spans="1:10" ht="24" customHeight="1">
+      <c r="A230" s="18" t="s"/>
+      <c r="B230" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C230" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D230" s="11" t="s"/>
+      <c r="E230" s="24" t="s"/>
+      <c r="F230" s="11" t="s"/>
+      <c r="G230" s="24" t="s"/>
+      <c r="H230" s="11" t="s"/>
+      <c r="I230" s="24" t="s"/>
+      <c r="J230" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="231" spans="1:10" ht="24" customHeight="1">
+      <c r="A231" s="18" t="s"/>
+      <c r="B231" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C231" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D231" s="11" t="s"/>
+      <c r="E231" s="24" t="s"/>
+      <c r="F231" s="11" t="s"/>
+      <c r="G231" s="24" t="s"/>
+      <c r="H231" s="11" t="s"/>
+      <c r="I231" s="24" t="s"/>
+      <c r="J231" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="232" spans="1:10" ht="24" customHeight="1">
+      <c r="A232" s="9" t="s"/>
+      <c r="B232" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C232" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D232" s="11" t="s"/>
+      <c r="E232" s="24" t="s"/>
+      <c r="F232" s="11" t="s"/>
+      <c r="G232" s="24" t="s"/>
+      <c r="H232" s="11" t="s"/>
+      <c r="I232" s="24" t="s"/>
+      <c r="J232" s="32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="233" spans="1:10" ht="24" customHeight="1">
+      <c r="A233" s="18" t="s"/>
+      <c r="B233" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C233" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D233" s="11" t="s"/>
+      <c r="E233" s="24" t="s"/>
+      <c r="F233" s="11" t="s"/>
+      <c r="G233" s="24" t="s"/>
+      <c r="H233" s="11" t="s"/>
+      <c r="I233" s="24" t="s"/>
+      <c r="J233" s="32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="234" spans="1:10" ht="24" customHeight="1">
+      <c r="A234" s="18" t="s"/>
+      <c r="B234" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C234" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D234" s="11" t="s"/>
+      <c r="E234" s="24" t="s"/>
+      <c r="F234" s="11" t="s"/>
+      <c r="G234" s="24" t="s"/>
+      <c r="H234" s="11" t="s"/>
+      <c r="I234" s="24" t="s"/>
+      <c r="J234" s="32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="235" spans="1:10" ht="24" customHeight="1">
+      <c r="A235" s="18" t="s"/>
+      <c r="B235" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C235" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D235" s="11" t="s"/>
+      <c r="E235" s="24" t="s"/>
+      <c r="F235" s="11" t="s"/>
+      <c r="G235" s="24" t="s"/>
+      <c r="H235" s="11" t="s"/>
+      <c r="I235" s="24" t="s"/>
+      <c r="J235" s="32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="236" spans="1:10" ht="24" customHeight="1">
+      <c r="A236" s="18" t="s"/>
+      <c r="B236" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C236" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D236" s="11" t="s"/>
+      <c r="E236" s="24" t="s"/>
+      <c r="F236" s="11" t="s"/>
+      <c r="G236" s="24" t="s"/>
+      <c r="H236" s="11" t="s"/>
+      <c r="I236" s="24" t="s"/>
+      <c r="J236" s="32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="237" spans="1:10" ht="24" customHeight="1">
+      <c r="A237" s="18" t="s"/>
+      <c r="B237" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C237" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D237" s="11" t="s"/>
+      <c r="E237" s="24" t="s"/>
+      <c r="F237" s="11" t="s"/>
+      <c r="G237" s="24" t="s"/>
+      <c r="H237" s="11" t="s"/>
+      <c r="I237" s="24" t="s"/>
+      <c r="J237" s="32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="238" spans="1:10" ht="24" customHeight="1">
+      <c r="A238" s="9" t="s"/>
+      <c r="B238" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C238" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D238" s="11" t="s"/>
+      <c r="E238" s="24" t="s"/>
+      <c r="F238" s="11" t="s"/>
+      <c r="G238" s="24" t="s"/>
+      <c r="H238" s="11" t="s"/>
+      <c r="I238" s="24" t="s"/>
+      <c r="J238" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="239" spans="1:10" ht="24" customHeight="1">
+      <c r="A239" s="18" t="s"/>
+      <c r="B239" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C239" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D239" s="11" t="s"/>
+      <c r="E239" s="24" t="s"/>
+      <c r="F239" s="11" t="s"/>
+      <c r="G239" s="24" t="s"/>
+      <c r="H239" s="11" t="s"/>
+      <c r="I239" s="24" t="s"/>
+      <c r="J239" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="240" spans="1:10" ht="24" customHeight="1">
+      <c r="A240" s="18" t="s"/>
+      <c r="B240" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C240" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D240" s="11" t="s"/>
+      <c r="E240" s="24" t="s"/>
+      <c r="F240" s="11" t="s"/>
+      <c r="G240" s="24" t="s"/>
+      <c r="H240" s="11" t="s"/>
+      <c r="I240" s="24" t="s"/>
+      <c r="J240" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="241" spans="1:10" ht="24" customHeight="1">
+      <c r="A241" s="18" t="s"/>
+      <c r="B241" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C241" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D241" s="11" t="s"/>
+      <c r="E241" s="24" t="s"/>
+      <c r="F241" s="11" t="s"/>
+      <c r="G241" s="24" t="s"/>
+      <c r="H241" s="11" t="s"/>
+      <c r="I241" s="24" t="s"/>
+      <c r="J241" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="242" spans="1:10" ht="24" customHeight="1">
+      <c r="A242" s="18" t="s"/>
+      <c r="B242" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C242" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D242" s="11" t="s"/>
+      <c r="E242" s="24" t="s"/>
+      <c r="F242" s="11" t="s"/>
+      <c r="G242" s="24" t="s"/>
+      <c r="H242" s="11" t="s"/>
+      <c r="I242" s="24" t="s"/>
+      <c r="J242" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="243" spans="1:10" ht="24" customHeight="1">
+      <c r="A243" s="18" t="s"/>
+      <c r="B243" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C243" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D243" s="11" t="s"/>
+      <c r="E243" s="24" t="s"/>
+      <c r="F243" s="11" t="s"/>
+      <c r="G243" s="24" t="s"/>
+      <c r="H243" s="11" t="s"/>
+      <c r="I243" s="24" t="s"/>
+      <c r="J243" s="32" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add bartender art and CharacterPart configuration
</commit_message>
<xml_diff>
--- a/Excel/CharacterPart.xlsx
+++ b/Excel/CharacterPart.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t/>
   </si>
@@ -284,6 +284,39 @@
   </si>
   <si>
     <t>character_c_sit_hair_03</t>
+  </si>
+  <si>
+    <t>character_c_idle_body_00m</t>
+  </si>
+  <si>
+    <t>character_c_idle_face_00</t>
+  </si>
+  <si>
+    <t>character_c_idle_hair_00</t>
+  </si>
+  <si>
+    <t>character_r_idle_hair_00</t>
+  </si>
+  <si>
+    <t>character_c_sit_body_00</t>
+  </si>
+  <si>
+    <t>character_c_sit_face_00</t>
+  </si>
+  <si>
+    <t>character_c_sit_hair_00</t>
+  </si>
+  <si>
+    <t>character_c_walk_body_00</t>
+  </si>
+  <si>
+    <t>character_c_walk_face_00</t>
+  </si>
+  <si>
+    <t>character_c_walk_hair_00</t>
+  </si>
+  <si>
+    <t>character_empty</t>
   </si>
 </sst>
 </file>
@@ -711,7 +744,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="J327"/>
+  <dimension ref="J393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.7109" customWidth="1"/>
@@ -6671,6 +6704,1110 @@
       <c r="I327" s="24" t="s"/>
       <c r="J327" s="32" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="328" spans="1:10" ht="24" customHeight="1">
+      <c r="A328" s="18" t="s"/>
+      <c r="B328" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C328" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D328" s="11" t="s"/>
+      <c r="E328" s="24" t="s"/>
+      <c r="F328" s="11" t="s"/>
+      <c r="G328" s="24" t="s"/>
+      <c r="H328" s="11" t="s"/>
+      <c r="I328" s="24" t="s"/>
+      <c r="J328" s="32" t="s"/>
+    </row>
+    <row r="329" spans="1:10" ht="24" customHeight="1">
+      <c r="A329" s="18" t="s"/>
+      <c r="B329" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C329" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D329" s="11" t="s"/>
+      <c r="E329" s="24" t="s"/>
+      <c r="F329" s="11" t="s"/>
+      <c r="G329" s="24" t="s"/>
+      <c r="H329" s="11" t="s"/>
+      <c r="I329" s="24" t="s"/>
+      <c r="J329" s="32" t="s"/>
+    </row>
+    <row r="330" spans="1:10" ht="24" customHeight="1">
+      <c r="A330" s="18" t="s"/>
+      <c r="B330" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C330" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D330" s="11" t="s"/>
+      <c r="E330" s="24" t="s"/>
+      <c r="F330" s="11" t="s"/>
+      <c r="G330" s="24" t="s"/>
+      <c r="H330" s="11" t="s"/>
+      <c r="I330" s="24" t="s"/>
+      <c r="J330" s="32" t="s"/>
+    </row>
+    <row r="331" spans="1:10" ht="24" customHeight="1">
+      <c r="A331" s="18" t="s"/>
+      <c r="B331" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C331" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D331" s="11" t="s"/>
+      <c r="E331" s="24" t="s"/>
+      <c r="F331" s="11" t="s"/>
+      <c r="G331" s="24" t="s"/>
+      <c r="H331" s="11" t="s"/>
+      <c r="I331" s="24" t="s"/>
+      <c r="J331" s="32" t="s"/>
+    </row>
+    <row r="332" spans="1:10" ht="24" customHeight="1">
+      <c r="A332" s="18" t="s"/>
+      <c r="B332" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C332" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D332" s="11" t="s"/>
+      <c r="E332" s="24" t="s"/>
+      <c r="F332" s="11" t="s"/>
+      <c r="G332" s="24" t="s"/>
+      <c r="H332" s="11" t="s"/>
+      <c r="I332" s="24" t="s"/>
+      <c r="J332" s="32" t="s"/>
+    </row>
+    <row r="333" spans="1:10" ht="24" customHeight="1">
+      <c r="A333" s="18" t="s"/>
+      <c r="B333" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C333" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D333" s="11" t="s"/>
+      <c r="E333" s="24" t="s"/>
+      <c r="F333" s="11" t="s"/>
+      <c r="G333" s="24" t="s"/>
+      <c r="H333" s="11" t="s"/>
+      <c r="I333" s="24" t="s"/>
+      <c r="J333" s="32" t="s"/>
+    </row>
+    <row r="334" spans="1:10" ht="24" customHeight="1">
+      <c r="A334" s="18" t="s"/>
+      <c r="B334" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C334" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D334" s="11" t="s"/>
+      <c r="E334" s="24" t="s"/>
+      <c r="F334" s="11" t="s"/>
+      <c r="G334" s="24" t="s"/>
+      <c r="H334" s="11" t="s"/>
+      <c r="I334" s="24" t="s"/>
+      <c r="J334" s="32" t="s"/>
+    </row>
+    <row r="335" spans="1:10" ht="24" customHeight="1">
+      <c r="A335" s="18" t="s"/>
+      <c r="B335" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C335" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D335" s="11" t="s"/>
+      <c r="E335" s="24" t="s"/>
+      <c r="F335" s="11" t="s"/>
+      <c r="G335" s="24" t="s"/>
+      <c r="H335" s="11" t="s"/>
+      <c r="I335" s="24" t="s"/>
+      <c r="J335" s="32" t="s"/>
+    </row>
+    <row r="336" spans="1:10" ht="24" customHeight="1">
+      <c r="A336" s="18" t="s"/>
+      <c r="B336" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C336" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D336" s="11" t="s"/>
+      <c r="E336" s="24" t="s"/>
+      <c r="F336" s="11" t="s"/>
+      <c r="G336" s="24" t="s"/>
+      <c r="H336" s="11" t="s"/>
+      <c r="I336" s="24" t="s"/>
+      <c r="J336" s="32" t="s"/>
+    </row>
+    <row r="337" spans="1:10" ht="24" customHeight="1">
+      <c r="A337" s="18" t="s"/>
+      <c r="B337" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C337" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D337" s="11" t="s"/>
+      <c r="E337" s="24" t="s"/>
+      <c r="F337" s="11" t="s"/>
+      <c r="G337" s="24" t="s"/>
+      <c r="H337" s="11" t="s"/>
+      <c r="I337" s="24" t="s"/>
+      <c r="J337" s="32" t="s"/>
+    </row>
+    <row r="338" spans="1:10" ht="24" customHeight="1">
+      <c r="A338" s="18" t="s"/>
+      <c r="B338" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C338" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D338" s="11" t="s"/>
+      <c r="E338" s="24" t="s"/>
+      <c r="F338" s="11" t="s"/>
+      <c r="G338" s="24" t="s"/>
+      <c r="H338" s="11" t="s"/>
+      <c r="I338" s="24" t="s"/>
+      <c r="J338" s="32" t="s"/>
+    </row>
+    <row r="339" spans="1:10" ht="24" customHeight="1">
+      <c r="A339" s="18" t="s"/>
+      <c r="B339" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C339" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D339" s="11" t="s"/>
+      <c r="E339" s="24" t="s"/>
+      <c r="F339" s="11" t="s"/>
+      <c r="G339" s="24" t="s"/>
+      <c r="H339" s="11" t="s"/>
+      <c r="I339" s="24" t="s"/>
+      <c r="J339" s="32" t="s"/>
+    </row>
+    <row r="340" spans="1:10" ht="24" customHeight="1">
+      <c r="A340" s="18" t="s"/>
+      <c r="B340" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C340" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D340" s="11" t="s"/>
+      <c r="E340" s="24" t="s"/>
+      <c r="F340" s="11" t="s"/>
+      <c r="G340" s="24" t="s"/>
+      <c r="H340" s="11" t="s"/>
+      <c r="I340" s="24" t="s"/>
+      <c r="J340" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="341" spans="1:10" ht="24" customHeight="1">
+      <c r="A341" s="18" t="s"/>
+      <c r="B341" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C341" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D341" s="11" t="s"/>
+      <c r="E341" s="24" t="s"/>
+      <c r="F341" s="11" t="s"/>
+      <c r="G341" s="24" t="s"/>
+      <c r="H341" s="11" t="s"/>
+      <c r="I341" s="24" t="s"/>
+      <c r="J341" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="342" spans="1:10" ht="24" customHeight="1">
+      <c r="A342" s="18" t="s"/>
+      <c r="B342" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C342" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D342" s="11" t="s"/>
+      <c r="E342" s="24" t="s"/>
+      <c r="F342" s="11" t="s"/>
+      <c r="G342" s="24" t="s"/>
+      <c r="H342" s="11" t="s"/>
+      <c r="I342" s="24" t="s"/>
+      <c r="J342" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="343" spans="1:10" ht="24" customHeight="1">
+      <c r="A343" s="18" t="s"/>
+      <c r="B343" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C343" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D343" s="11" t="s"/>
+      <c r="E343" s="24" t="s"/>
+      <c r="F343" s="11" t="s"/>
+      <c r="G343" s="24" t="s"/>
+      <c r="H343" s="11" t="s"/>
+      <c r="I343" s="24" t="s"/>
+      <c r="J343" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="344" spans="1:10" ht="24" customHeight="1">
+      <c r="A344" s="18" t="s"/>
+      <c r="B344" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C344" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D344" s="11" t="s"/>
+      <c r="E344" s="24" t="s"/>
+      <c r="F344" s="11" t="s"/>
+      <c r="G344" s="24" t="s"/>
+      <c r="H344" s="11" t="s"/>
+      <c r="I344" s="24" t="s"/>
+      <c r="J344" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="345" spans="1:10" ht="24" customHeight="1">
+      <c r="A345" s="18" t="s"/>
+      <c r="B345" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C345" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D345" s="11" t="s"/>
+      <c r="E345" s="24" t="s"/>
+      <c r="F345" s="11" t="s"/>
+      <c r="G345" s="24" t="s"/>
+      <c r="H345" s="11" t="s"/>
+      <c r="I345" s="24" t="s"/>
+      <c r="J345" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="346" spans="1:10" ht="24" customHeight="1">
+      <c r="A346" s="18" t="s"/>
+      <c r="B346" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C346" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D346" s="11" t="s"/>
+      <c r="E346" s="24" t="s"/>
+      <c r="F346" s="11" t="s"/>
+      <c r="G346" s="24" t="s"/>
+      <c r="H346" s="11" t="s"/>
+      <c r="I346" s="24" t="s"/>
+      <c r="J346" s="32" t="s"/>
+    </row>
+    <row r="347" spans="1:10" ht="24" customHeight="1">
+      <c r="A347" s="18" t="s"/>
+      <c r="B347" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C347" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D347" s="11" t="s"/>
+      <c r="E347" s="24" t="s"/>
+      <c r="F347" s="11" t="s"/>
+      <c r="G347" s="24" t="s"/>
+      <c r="H347" s="11" t="s"/>
+      <c r="I347" s="24" t="s"/>
+      <c r="J347" s="32" t="s"/>
+    </row>
+    <row r="348" spans="1:10" ht="24" customHeight="1">
+      <c r="A348" s="18" t="s"/>
+      <c r="B348" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C348" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D348" s="11" t="s"/>
+      <c r="E348" s="24" t="s"/>
+      <c r="F348" s="11" t="s"/>
+      <c r="G348" s="24" t="s"/>
+      <c r="H348" s="11" t="s"/>
+      <c r="I348" s="24" t="s"/>
+      <c r="J348" s="32" t="s"/>
+    </row>
+    <row r="349" spans="1:10" ht="24" customHeight="1">
+      <c r="A349" s="18" t="s"/>
+      <c r="B349" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C349" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D349" s="11" t="s"/>
+      <c r="E349" s="24" t="s"/>
+      <c r="F349" s="11" t="s"/>
+      <c r="G349" s="24" t="s"/>
+      <c r="H349" s="11" t="s"/>
+      <c r="I349" s="24" t="s"/>
+      <c r="J349" s="32" t="s"/>
+    </row>
+    <row r="350" spans="1:10" ht="24" customHeight="1">
+      <c r="A350" s="18" t="s"/>
+      <c r="B350" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C350" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D350" s="11" t="s"/>
+      <c r="E350" s="24" t="s"/>
+      <c r="F350" s="11" t="s"/>
+      <c r="G350" s="24" t="s"/>
+      <c r="H350" s="11" t="s"/>
+      <c r="I350" s="24" t="s"/>
+      <c r="J350" s="32" t="s"/>
+    </row>
+    <row r="351" spans="1:10" ht="24" customHeight="1">
+      <c r="A351" s="18" t="s"/>
+      <c r="B351" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C351" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D351" s="11" t="s"/>
+      <c r="E351" s="24" t="s"/>
+      <c r="F351" s="11" t="s"/>
+      <c r="G351" s="24" t="s"/>
+      <c r="H351" s="11" t="s"/>
+      <c r="I351" s="24" t="s"/>
+      <c r="J351" s="32" t="s"/>
+    </row>
+    <row r="352" spans="1:10" ht="24" customHeight="1">
+      <c r="A352" s="18" t="s"/>
+      <c r="B352" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C352" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D352" s="11" t="s"/>
+      <c r="E352" s="24" t="s"/>
+      <c r="F352" s="11" t="s"/>
+      <c r="G352" s="24" t="s"/>
+      <c r="H352" s="11" t="s"/>
+      <c r="I352" s="24" t="s"/>
+      <c r="J352" s="32" t="s"/>
+    </row>
+    <row r="353" spans="1:10" ht="24" customHeight="1">
+      <c r="A353" s="18" t="s"/>
+      <c r="B353" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C353" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D353" s="11" t="s"/>
+      <c r="E353" s="24" t="s"/>
+      <c r="F353" s="11" t="s"/>
+      <c r="G353" s="24" t="s"/>
+      <c r="H353" s="11" t="s"/>
+      <c r="I353" s="24" t="s"/>
+      <c r="J353" s="32" t="s"/>
+    </row>
+    <row r="354" spans="1:10" ht="24" customHeight="1">
+      <c r="A354" s="18" t="s"/>
+      <c r="B354" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C354" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D354" s="11" t="s"/>
+      <c r="E354" s="24" t="s"/>
+      <c r="F354" s="11" t="s"/>
+      <c r="G354" s="24" t="s"/>
+      <c r="H354" s="11" t="s"/>
+      <c r="I354" s="24" t="s"/>
+      <c r="J354" s="32" t="s"/>
+    </row>
+    <row r="355" spans="1:10" ht="24" customHeight="1">
+      <c r="A355" s="18" t="s"/>
+      <c r="B355" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C355" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D355" s="11" t="s"/>
+      <c r="E355" s="24" t="s"/>
+      <c r="F355" s="11" t="s"/>
+      <c r="G355" s="24" t="s"/>
+      <c r="H355" s="11" t="s"/>
+      <c r="I355" s="24" t="s"/>
+      <c r="J355" s="32" t="s"/>
+    </row>
+    <row r="356" spans="1:10" ht="24" customHeight="1">
+      <c r="A356" s="18" t="s"/>
+      <c r="B356" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C356" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D356" s="11" t="s"/>
+      <c r="E356" s="24" t="s"/>
+      <c r="F356" s="11" t="s"/>
+      <c r="G356" s="24" t="s"/>
+      <c r="H356" s="11" t="s"/>
+      <c r="I356" s="24" t="s"/>
+      <c r="J356" s="32" t="s"/>
+    </row>
+    <row r="357" spans="1:10" ht="24" customHeight="1">
+      <c r="A357" s="18" t="s"/>
+      <c r="B357" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C357" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D357" s="11" t="s"/>
+      <c r="E357" s="24" t="s"/>
+      <c r="F357" s="11" t="s"/>
+      <c r="G357" s="24" t="s"/>
+      <c r="H357" s="11" t="s"/>
+      <c r="I357" s="24" t="s"/>
+      <c r="J357" s="32" t="s"/>
+    </row>
+    <row r="358" spans="1:10" ht="24" customHeight="1">
+      <c r="A358" s="18" t="s"/>
+      <c r="B358" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C358" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D358" s="11" t="s"/>
+      <c r="E358" s="24" t="s"/>
+      <c r="F358" s="11" t="s"/>
+      <c r="G358" s="24" t="s"/>
+      <c r="H358" s="11" t="s"/>
+      <c r="I358" s="24" t="s"/>
+      <c r="J358" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="359" spans="1:10" ht="24" customHeight="1">
+      <c r="A359" s="18" t="s"/>
+      <c r="B359" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C359" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D359" s="11" t="s"/>
+      <c r="E359" s="24" t="s"/>
+      <c r="F359" s="11" t="s"/>
+      <c r="G359" s="24" t="s"/>
+      <c r="H359" s="11" t="s"/>
+      <c r="I359" s="24" t="s"/>
+      <c r="J359" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="360" spans="1:10" ht="24" customHeight="1">
+      <c r="A360" s="18" t="s"/>
+      <c r="B360" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C360" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D360" s="11" t="s"/>
+      <c r="E360" s="24" t="s"/>
+      <c r="F360" s="11" t="s"/>
+      <c r="G360" s="24" t="s"/>
+      <c r="H360" s="11" t="s"/>
+      <c r="I360" s="24" t="s"/>
+      <c r="J360" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="361" spans="1:10" ht="24" customHeight="1">
+      <c r="A361" s="18" t="s"/>
+      <c r="B361" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C361" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D361" s="11" t="s"/>
+      <c r="E361" s="24" t="s"/>
+      <c r="F361" s="11" t="s"/>
+      <c r="G361" s="24" t="s"/>
+      <c r="H361" s="11" t="s"/>
+      <c r="I361" s="24" t="s"/>
+      <c r="J361" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="362" spans="1:10" ht="24" customHeight="1">
+      <c r="A362" s="18" t="s"/>
+      <c r="B362" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C362" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D362" s="11" t="s"/>
+      <c r="E362" s="24" t="s"/>
+      <c r="F362" s="11" t="s"/>
+      <c r="G362" s="24" t="s"/>
+      <c r="H362" s="11" t="s"/>
+      <c r="I362" s="24" t="s"/>
+      <c r="J362" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="363" spans="1:10" ht="24" customHeight="1">
+      <c r="A363" s="18" t="s"/>
+      <c r="B363" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C363" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D363" s="11" t="s"/>
+      <c r="E363" s="24" t="s"/>
+      <c r="F363" s="11" t="s"/>
+      <c r="G363" s="24" t="s"/>
+      <c r="H363" s="11" t="s"/>
+      <c r="I363" s="24" t="s"/>
+      <c r="J363" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="364" spans="1:10" ht="24" customHeight="1">
+      <c r="A364" s="18" t="s"/>
+      <c r="B364" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C364" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D364" s="11" t="s"/>
+      <c r="E364" s="24" t="s"/>
+      <c r="F364" s="11" t="s"/>
+      <c r="G364" s="24" t="s"/>
+      <c r="H364" s="11" t="s"/>
+      <c r="I364" s="24" t="s"/>
+      <c r="J364" s="32" t="s"/>
+    </row>
+    <row r="365" spans="1:10" ht="24" customHeight="1">
+      <c r="A365" s="18" t="s"/>
+      <c r="B365" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C365" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D365" s="11" t="s"/>
+      <c r="E365" s="24" t="s"/>
+      <c r="F365" s="11" t="s"/>
+      <c r="G365" s="24" t="s"/>
+      <c r="H365" s="11" t="s"/>
+      <c r="I365" s="24" t="s"/>
+      <c r="J365" s="32" t="s"/>
+    </row>
+    <row r="366" spans="1:10" ht="24" customHeight="1">
+      <c r="A366" s="18" t="s"/>
+      <c r="B366" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C366" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D366" s="11" t="s"/>
+      <c r="E366" s="24" t="s"/>
+      <c r="F366" s="11" t="s"/>
+      <c r="G366" s="24" t="s"/>
+      <c r="H366" s="11" t="s"/>
+      <c r="I366" s="24" t="s"/>
+      <c r="J366" s="32" t="s"/>
+    </row>
+    <row r="367" spans="1:10" ht="24" customHeight="1">
+      <c r="A367" s="18" t="s"/>
+      <c r="B367" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C367" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D367" s="11" t="s"/>
+      <c r="E367" s="24" t="s"/>
+      <c r="F367" s="11" t="s"/>
+      <c r="G367" s="24" t="s"/>
+      <c r="H367" s="11" t="s"/>
+      <c r="I367" s="24" t="s"/>
+      <c r="J367" s="32" t="s"/>
+    </row>
+    <row r="368" spans="1:10" ht="24" customHeight="1">
+      <c r="A368" s="18" t="s"/>
+      <c r="B368" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C368" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D368" s="11" t="s"/>
+      <c r="E368" s="24" t="s"/>
+      <c r="F368" s="11" t="s"/>
+      <c r="G368" s="24" t="s"/>
+      <c r="H368" s="11" t="s"/>
+      <c r="I368" s="24" t="s"/>
+      <c r="J368" s="32" t="s"/>
+    </row>
+    <row r="369" spans="1:10" ht="24" customHeight="1">
+      <c r="A369" s="18" t="s"/>
+      <c r="B369" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C369" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D369" s="11" t="s"/>
+      <c r="E369" s="24" t="s"/>
+      <c r="F369" s="11" t="s"/>
+      <c r="G369" s="24" t="s"/>
+      <c r="H369" s="11" t="s"/>
+      <c r="I369" s="24" t="s"/>
+      <c r="J369" s="32" t="s"/>
+    </row>
+    <row r="370" spans="1:10" ht="24" customHeight="1">
+      <c r="A370" s="18" t="s"/>
+      <c r="B370" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C370" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D370" s="11" t="s"/>
+      <c r="E370" s="24" t="s"/>
+      <c r="F370" s="11" t="s"/>
+      <c r="G370" s="24" t="s"/>
+      <c r="H370" s="11" t="s"/>
+      <c r="I370" s="24" t="s"/>
+      <c r="J370" s="32" t="s"/>
+    </row>
+    <row r="371" spans="1:10" ht="24" customHeight="1">
+      <c r="A371" s="18" t="s"/>
+      <c r="B371" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C371" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D371" s="11" t="s"/>
+      <c r="E371" s="24" t="s"/>
+      <c r="F371" s="11" t="s"/>
+      <c r="G371" s="24" t="s"/>
+      <c r="H371" s="11" t="s"/>
+      <c r="I371" s="24" t="s"/>
+      <c r="J371" s="32" t="s"/>
+    </row>
+    <row r="372" spans="1:10" ht="24" customHeight="1">
+      <c r="A372" s="18" t="s"/>
+      <c r="B372" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C372" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D372" s="11" t="s"/>
+      <c r="E372" s="24" t="s"/>
+      <c r="F372" s="11" t="s"/>
+      <c r="G372" s="24" t="s"/>
+      <c r="H372" s="11" t="s"/>
+      <c r="I372" s="24" t="s"/>
+      <c r="J372" s="32" t="s"/>
+    </row>
+    <row r="373" spans="1:10" ht="24" customHeight="1">
+      <c r="A373" s="18" t="s"/>
+      <c r="B373" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C373" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D373" s="11" t="s"/>
+      <c r="E373" s="24" t="s"/>
+      <c r="F373" s="11" t="s"/>
+      <c r="G373" s="24" t="s"/>
+      <c r="H373" s="11" t="s"/>
+      <c r="I373" s="24" t="s"/>
+      <c r="J373" s="32" t="s"/>
+    </row>
+    <row r="374" spans="1:10" ht="24" customHeight="1">
+      <c r="A374" s="18" t="s"/>
+      <c r="B374" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C374" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D374" s="11" t="s"/>
+      <c r="E374" s="24" t="s"/>
+      <c r="F374" s="11" t="s"/>
+      <c r="G374" s="24" t="s"/>
+      <c r="H374" s="11" t="s"/>
+      <c r="I374" s="24" t="s"/>
+      <c r="J374" s="32" t="s"/>
+    </row>
+    <row r="375" spans="1:10" ht="24" customHeight="1">
+      <c r="A375" s="18" t="s"/>
+      <c r="B375" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C375" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D375" s="11" t="s"/>
+      <c r="E375" s="24" t="s"/>
+      <c r="F375" s="11" t="s"/>
+      <c r="G375" s="24" t="s"/>
+      <c r="H375" s="11" t="s"/>
+      <c r="I375" s="24" t="s"/>
+      <c r="J375" s="32" t="s"/>
+    </row>
+    <row r="376" spans="1:10" ht="24" customHeight="1">
+      <c r="A376" s="18" t="s"/>
+      <c r="B376" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C376" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D376" s="11" t="s"/>
+      <c r="E376" s="24" t="s"/>
+      <c r="F376" s="11" t="s"/>
+      <c r="G376" s="24" t="s"/>
+      <c r="H376" s="11" t="s"/>
+      <c r="I376" s="24" t="s"/>
+      <c r="J376" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="377" spans="1:10" ht="24" customHeight="1">
+      <c r="A377" s="18" t="s"/>
+      <c r="B377" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C377" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D377" s="11" t="s"/>
+      <c r="E377" s="24" t="s"/>
+      <c r="F377" s="11" t="s"/>
+      <c r="G377" s="24" t="s"/>
+      <c r="H377" s="11" t="s"/>
+      <c r="I377" s="24" t="s"/>
+      <c r="J377" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="378" spans="1:10" ht="24" customHeight="1">
+      <c r="A378" s="18" t="s"/>
+      <c r="B378" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C378" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D378" s="11" t="s"/>
+      <c r="E378" s="24" t="s"/>
+      <c r="F378" s="11" t="s"/>
+      <c r="G378" s="24" t="s"/>
+      <c r="H378" s="11" t="s"/>
+      <c r="I378" s="24" t="s"/>
+      <c r="J378" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="379" spans="1:10" ht="24" customHeight="1">
+      <c r="A379" s="18" t="s"/>
+      <c r="B379" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C379" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D379" s="11" t="s"/>
+      <c r="E379" s="24" t="s"/>
+      <c r="F379" s="11" t="s"/>
+      <c r="G379" s="24" t="s"/>
+      <c r="H379" s="11" t="s"/>
+      <c r="I379" s="24" t="s"/>
+      <c r="J379" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="380" spans="1:10" ht="24" customHeight="1">
+      <c r="A380" s="18" t="s"/>
+      <c r="B380" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C380" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D380" s="11" t="s"/>
+      <c r="E380" s="24" t="s"/>
+      <c r="F380" s="11" t="s"/>
+      <c r="G380" s="24" t="s"/>
+      <c r="H380" s="11" t="s"/>
+      <c r="I380" s="24" t="s"/>
+      <c r="J380" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="381" spans="1:10" ht="24" customHeight="1">
+      <c r="A381" s="18" t="s"/>
+      <c r="B381" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C381" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D381" s="11" t="s"/>
+      <c r="E381" s="24" t="s"/>
+      <c r="F381" s="11" t="s"/>
+      <c r="G381" s="24" t="s"/>
+      <c r="H381" s="11" t="s"/>
+      <c r="I381" s="24" t="s"/>
+      <c r="J381" s="32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="382" spans="1:10" ht="24" customHeight="1">
+      <c r="A382" s="18" t="s"/>
+      <c r="B382" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C382" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D382" s="11" t="s"/>
+      <c r="E382" s="24" t="s"/>
+      <c r="F382" s="11" t="s"/>
+      <c r="G382" s="24" t="s"/>
+      <c r="H382" s="11" t="s"/>
+      <c r="I382" s="24" t="s"/>
+      <c r="J382" s="32" t="s"/>
+    </row>
+    <row r="383" spans="1:10" ht="24" customHeight="1">
+      <c r="A383" s="18" t="s"/>
+      <c r="B383" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C383" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D383" s="11" t="s"/>
+      <c r="E383" s="24" t="s"/>
+      <c r="F383" s="11" t="s"/>
+      <c r="G383" s="24" t="s"/>
+      <c r="H383" s="11" t="s"/>
+      <c r="I383" s="24" t="s"/>
+      <c r="J383" s="32" t="s"/>
+    </row>
+    <row r="384" spans="1:10" ht="24" customHeight="1">
+      <c r="A384" s="18" t="s"/>
+      <c r="B384" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C384" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D384" s="11" t="s"/>
+      <c r="E384" s="24" t="s"/>
+      <c r="F384" s="11" t="s"/>
+      <c r="G384" s="24" t="s"/>
+      <c r="H384" s="11" t="s"/>
+      <c r="I384" s="24" t="s"/>
+      <c r="J384" s="32" t="s"/>
+    </row>
+    <row r="385" spans="1:10" ht="24" customHeight="1">
+      <c r="A385" s="18" t="s"/>
+      <c r="B385" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C385" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D385" s="11" t="s"/>
+      <c r="E385" s="24" t="s"/>
+      <c r="F385" s="11" t="s"/>
+      <c r="G385" s="24" t="s"/>
+      <c r="H385" s="11" t="s"/>
+      <c r="I385" s="24" t="s"/>
+      <c r="J385" s="32" t="s"/>
+    </row>
+    <row r="386" spans="1:10" ht="24" customHeight="1">
+      <c r="A386" s="18" t="s"/>
+      <c r="B386" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C386" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D386" s="11" t="s"/>
+      <c r="E386" s="24" t="s"/>
+      <c r="F386" s="11" t="s"/>
+      <c r="G386" s="24" t="s"/>
+      <c r="H386" s="11" t="s"/>
+      <c r="I386" s="24" t="s"/>
+      <c r="J386" s="32" t="s"/>
+    </row>
+    <row r="387" spans="1:10" ht="24" customHeight="1">
+      <c r="A387" s="18" t="s"/>
+      <c r="B387" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C387" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D387" s="11" t="s"/>
+      <c r="E387" s="24" t="s"/>
+      <c r="F387" s="11" t="s"/>
+      <c r="G387" s="24" t="s"/>
+      <c r="H387" s="11" t="s"/>
+      <c r="I387" s="24" t="s"/>
+      <c r="J387" s="32" t="s"/>
+    </row>
+    <row r="388" spans="1:10" ht="24" customHeight="1">
+      <c r="A388" s="18" t="s"/>
+      <c r="B388" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C388" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D388" s="11" t="s"/>
+      <c r="E388" s="24" t="s"/>
+      <c r="F388" s="11" t="s"/>
+      <c r="G388" s="24" t="s"/>
+      <c r="H388" s="11" t="s"/>
+      <c r="I388" s="24" t="s"/>
+      <c r="J388" s="32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="389" spans="1:10" ht="24" customHeight="1">
+      <c r="A389" s="18" t="s"/>
+      <c r="B389" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C389" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D389" s="11" t="s"/>
+      <c r="E389" s="24" t="s"/>
+      <c r="F389" s="11" t="s"/>
+      <c r="G389" s="24" t="s"/>
+      <c r="H389" s="11" t="s"/>
+      <c r="I389" s="24" t="s"/>
+      <c r="J389" s="32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="390" spans="1:10" ht="24" customHeight="1">
+      <c r="A390" s="18" t="s"/>
+      <c r="B390" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C390" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D390" s="11" t="s"/>
+      <c r="E390" s="24" t="s"/>
+      <c r="F390" s="11" t="s"/>
+      <c r="G390" s="24" t="s"/>
+      <c r="H390" s="11" t="s"/>
+      <c r="I390" s="24" t="s"/>
+      <c r="J390" s="32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="391" spans="1:10" ht="24" customHeight="1">
+      <c r="A391" s="18" t="s"/>
+      <c r="B391" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C391" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D391" s="11" t="s"/>
+      <c r="E391" s="24" t="s"/>
+      <c r="F391" s="11" t="s"/>
+      <c r="G391" s="24" t="s"/>
+      <c r="H391" s="11" t="s"/>
+      <c r="I391" s="24" t="s"/>
+      <c r="J391" s="32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="392" spans="1:10" ht="24" customHeight="1">
+      <c r="A392" s="18" t="s"/>
+      <c r="B392" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C392" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D392" s="11" t="s"/>
+      <c r="E392" s="24" t="s"/>
+      <c r="F392" s="11" t="s"/>
+      <c r="G392" s="24" t="s"/>
+      <c r="H392" s="11" t="s"/>
+      <c r="I392" s="24" t="s"/>
+      <c r="J392" s="32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="393" spans="1:10" ht="24" customHeight="1">
+      <c r="A393" s="18" t="s"/>
+      <c r="B393" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C393" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D393" s="11" t="s"/>
+      <c r="E393" s="24" t="s"/>
+      <c r="F393" s="11" t="s"/>
+      <c r="G393" s="24" t="s"/>
+      <c r="H393" s="11" t="s"/>
+      <c r="I393" s="24" t="s"/>
+      <c r="J393" s="32" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync remaining character body art and CharacterPart entries
</commit_message>
<xml_diff>
--- a/Excel/CharacterPart.xlsx
+++ b/Excel/CharacterPart.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t/>
   </si>
@@ -317,6 +317,12 @@
   </si>
   <si>
     <t>character_empty</t>
+  </si>
+  <si>
+    <t>character_c_walk_body_02</t>
+  </si>
+  <si>
+    <t>character_c_sit_body_02</t>
   </si>
 </sst>
 </file>
@@ -744,7 +750,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="J393"/>
+  <dimension ref="J405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.7109" customWidth="1"/>
@@ -7808,6 +7814,222 @@
       <c r="I393" s="24" t="s"/>
       <c r="J393" s="32" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="394" spans="1:10" ht="24" customHeight="1">
+      <c r="A394" s="18" t="s"/>
+      <c r="B394" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C394" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D394" s="11" t="s"/>
+      <c r="E394" s="24" t="s"/>
+      <c r="F394" s="11" t="s"/>
+      <c r="G394" s="24" t="s"/>
+      <c r="H394" s="11" t="s"/>
+      <c r="I394" s="24" t="s"/>
+      <c r="J394" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="395" spans="1:10" ht="24" customHeight="1">
+      <c r="A395" s="18" t="s"/>
+      <c r="B395" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C395" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D395" s="11" t="s"/>
+      <c r="E395" s="24" t="s"/>
+      <c r="F395" s="11" t="s"/>
+      <c r="G395" s="24" t="s"/>
+      <c r="H395" s="11" t="s"/>
+      <c r="I395" s="24" t="s"/>
+      <c r="J395" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="396" spans="1:10" ht="24" customHeight="1">
+      <c r="A396" s="18" t="s"/>
+      <c r="B396" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C396" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D396" s="11" t="s"/>
+      <c r="E396" s="24" t="s"/>
+      <c r="F396" s="11" t="s"/>
+      <c r="G396" s="24" t="s"/>
+      <c r="H396" s="11" t="s"/>
+      <c r="I396" s="24" t="s"/>
+      <c r="J396" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="397" spans="1:10" ht="24" customHeight="1">
+      <c r="A397" s="18" t="s"/>
+      <c r="B397" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C397" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D397" s="11" t="s"/>
+      <c r="E397" s="24" t="s"/>
+      <c r="F397" s="11" t="s"/>
+      <c r="G397" s="24" t="s"/>
+      <c r="H397" s="11" t="s"/>
+      <c r="I397" s="24" t="s"/>
+      <c r="J397" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="398" spans="1:10" ht="24" customHeight="1">
+      <c r="A398" s="18" t="s"/>
+      <c r="B398" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C398" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D398" s="11" t="s"/>
+      <c r="E398" s="24" t="s"/>
+      <c r="F398" s="11" t="s"/>
+      <c r="G398" s="24" t="s"/>
+      <c r="H398" s="11" t="s"/>
+      <c r="I398" s="24" t="s"/>
+      <c r="J398" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="399" spans="1:10" ht="24" customHeight="1">
+      <c r="A399" s="18" t="s"/>
+      <c r="B399" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C399" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D399" s="11" t="s"/>
+      <c r="E399" s="24" t="s"/>
+      <c r="F399" s="11" t="s"/>
+      <c r="G399" s="24" t="s"/>
+      <c r="H399" s="11" t="s"/>
+      <c r="I399" s="24" t="s"/>
+      <c r="J399" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="400" spans="1:10" ht="24" customHeight="1">
+      <c r="A400" s="18" t="s"/>
+      <c r="B400" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C400" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D400" s="11" t="s"/>
+      <c r="E400" s="24" t="s"/>
+      <c r="F400" s="11" t="s"/>
+      <c r="G400" s="24" t="s"/>
+      <c r="H400" s="11" t="s"/>
+      <c r="I400" s="24" t="s"/>
+      <c r="J400" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="401" spans="1:10" ht="24" customHeight="1">
+      <c r="A401" s="18" t="s"/>
+      <c r="B401" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C401" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D401" s="11" t="s"/>
+      <c r="E401" s="24" t="s"/>
+      <c r="F401" s="11" t="s"/>
+      <c r="G401" s="24" t="s"/>
+      <c r="H401" s="11" t="s"/>
+      <c r="I401" s="24" t="s"/>
+      <c r="J401" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="402" spans="1:10" ht="24" customHeight="1">
+      <c r="A402" s="18" t="s"/>
+      <c r="B402" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C402" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D402" s="11" t="s"/>
+      <c r="E402" s="24" t="s"/>
+      <c r="F402" s="11" t="s"/>
+      <c r="G402" s="24" t="s"/>
+      <c r="H402" s="11" t="s"/>
+      <c r="I402" s="24" t="s"/>
+      <c r="J402" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="403" spans="1:10" ht="24" customHeight="1">
+      <c r="A403" s="18" t="s"/>
+      <c r="B403" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C403" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D403" s="11" t="s"/>
+      <c r="E403" s="24" t="s"/>
+      <c r="F403" s="11" t="s"/>
+      <c r="G403" s="24" t="s"/>
+      <c r="H403" s="11" t="s"/>
+      <c r="I403" s="24" t="s"/>
+      <c r="J403" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="404" spans="1:10" ht="24" customHeight="1">
+      <c r="A404" s="18" t="s"/>
+      <c r="B404" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C404" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D404" s="11" t="s"/>
+      <c r="E404" s="24" t="s"/>
+      <c r="F404" s="11" t="s"/>
+      <c r="G404" s="24" t="s"/>
+      <c r="H404" s="11" t="s"/>
+      <c r="I404" s="24" t="s"/>
+      <c r="J404" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="405" spans="1:10" ht="24" customHeight="1">
+      <c r="A405" s="18" t="s"/>
+      <c r="B405" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C405" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D405" s="11" t="s"/>
+      <c r="E405" s="24" t="s"/>
+      <c r="F405" s="11" t="s"/>
+      <c r="G405" s="24" t="s"/>
+      <c r="H405" s="11" t="s"/>
+      <c r="I405" s="24" t="s"/>
+      <c r="J405" s="32" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>